<commit_message>
Update documentation and insights
</commit_message>
<xml_diff>
--- a/01_database/05_data_dictionary.xlsx
+++ b/01_database/05_data_dictionary.xlsx
@@ -8,22 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Data analys plan\Dứa Data Learning\Banking-Performance-Analytics\01_database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9E6A937F-EDBA-4A59-AA3F-9D46E054BB48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD68C702-623C-4D9C-8FCE-534C3A396ABD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" firstSheet="3" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="0" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="01_Table_Overview" sheetId="1" r:id="rId1"/>
     <sheet name="02_Column_Dictionary" sheetId="2" r:id="rId2"/>
     <sheet name="03_Relationships" sheetId="3" r:id="rId3"/>
     <sheet name="04_SQL_Views" sheetId="4" r:id="rId4"/>
-    <sheet name="05_DAX_Measures" sheetId="5" r:id="rId5"/>
-    <sheet name="06_Dashboard_Mapping" sheetId="6" r:id="rId6"/>
+    <sheet name="06_Dashboard_Mapping" sheetId="6" r:id="rId5"/>
+    <sheet name="05_DAX_Measures" sheetId="5" r:id="rId6"/>
     <sheet name="07_Data_Quality_Checks" sheetId="7" r:id="rId7"/>
     <sheet name="08_Source_Files" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="0"/>
-  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
@@ -1955,19 +1954,6 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="05_DAX_MeasuresTable" displayName="_05_DAX_MeasuresTable" ref="A4:E28">
-  <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="Measure Name"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="DAX Formula"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="Business Meaning"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0400-000004000000}" name="Format"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0400-000005000000}" name="Dashboard Page"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="06_Dashboard_MappingTable" displayName="_06_Dashboard_MappingTable" ref="A4:F26">
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" name="Dashboard Page"/>
@@ -1976,6 +1962,19 @@
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0500-000004000000}" name="Main Fields / Measures"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0500-000005000000}" name="Source View / Table"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0500-000006000000}" name="Business Question"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="05_DAX_MeasuresTable" displayName="_05_DAX_MeasuresTable" ref="A4:E28">
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="Measure Name"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="DAX Formula"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="Business Meaning"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0400-000004000000}" name="Format"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0400-000005000000}" name="Dashboard Page"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5680,482 +5679,6 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:E28"/>
-  <sheetFormatPr defaultRowHeight="14"/>
-  <cols>
-    <col min="1" max="1" width="34" customWidth="1"/>
-    <col min="2" max="2" width="88" customWidth="1"/>
-    <col min="3" max="3" width="66" customWidth="1"/>
-    <col min="4" max="4" width="18" customWidth="1"/>
-    <col min="5" max="5" width="34" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" ht="17.399999999999999" customHeight="1">
-      <c r="A1" s="4" t="s">
-        <v>363</v>
-      </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-    </row>
-    <row r="2" spans="1:5" ht="13.4" customHeight="1">
-      <c r="A2" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-    </row>
-    <row r="3" spans="1:5" ht="58">
-      <c r="A3" s="3" t="s">
-        <v>364</v>
-      </c>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-    </row>
-    <row r="4" spans="1:5" ht="16.649999999999999" customHeight="1">
-      <c r="A4" s="1" t="s">
-        <v>365</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>366</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>281</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>367</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>368</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5">
-      <c r="A5" s="2" t="s">
-        <v>369</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>370</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>371</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>372</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>373</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5">
-      <c r="A6" s="2" t="s">
-        <v>374</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>375</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>376</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>372</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5">
-      <c r="A7" s="2" t="s">
-        <v>377</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>378</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>379</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>372</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5">
-      <c r="A8" s="2" t="s">
-        <v>380</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>381</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>382</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>383</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5">
-      <c r="A9" s="2" t="s">
-        <v>384</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>385</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>386</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>383</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5">
-      <c r="A10" s="2" t="s">
-        <v>387</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>388</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>389</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>383</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5">
-      <c r="A11" s="2" t="s">
-        <v>391</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>392</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>393</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>383</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="25">
-      <c r="A12" s="2" t="s">
-        <v>394</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>395</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>396</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>397</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5">
-      <c r="A13" s="2" t="s">
-        <v>398</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>399</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>400</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>383</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>401</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5">
-      <c r="A14" s="2" t="s">
-        <v>402</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>403</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>404</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>372</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5">
-      <c r="A15" s="2" t="s">
-        <v>406</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>407</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>408</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>383</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" ht="25">
-      <c r="A16" s="2" t="s">
-        <v>409</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>410</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>411</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>397</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5">
-      <c r="A17" s="2" t="s">
-        <v>412</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>413</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>414</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>383</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>401</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5">
-      <c r="A18" s="2" t="s">
-        <v>415</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>416</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>417</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>397</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>401</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5">
-      <c r="A19" s="2" t="s">
-        <v>418</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>419</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>420</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>383</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>421</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5">
-      <c r="A20" s="2" t="s">
-        <v>422</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>423</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>424</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>383</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5">
-      <c r="A21" s="2" t="s">
-        <v>425</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>426</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>427</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>383</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" ht="25">
-      <c r="A22" s="2" t="s">
-        <v>428</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>429</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>430</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>383</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5">
-      <c r="A23" s="2" t="s">
-        <v>432</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>433</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>397</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" ht="25">
-      <c r="A24" s="2" t="s">
-        <v>435</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>436</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>437</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>372</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5">
-      <c r="A25" s="2" t="s">
-        <v>438</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>439</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>440</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>383</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>441</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5">
-      <c r="A26" s="2" t="s">
-        <v>442</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>443</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>444</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>397</v>
-      </c>
-      <c r="E26" s="2" t="s">
-        <v>441</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" ht="25">
-      <c r="A27" s="2" t="s">
-        <v>445</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>446</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>447</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>372</v>
-      </c>
-      <c r="E27" s="2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" ht="25">
-      <c r="A28" s="2" t="s">
-        <v>448</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>449</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>450</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>383</v>
-      </c>
-      <c r="E28" s="2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A2:E2"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:F26"/>
   <sheetFormatPr defaultRowHeight="14"/>
@@ -6652,6 +6175,482 @@
   <mergeCells count="2">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <dimension ref="A1:E28"/>
+  <sheetFormatPr defaultRowHeight="14"/>
+  <cols>
+    <col min="1" max="1" width="34" customWidth="1"/>
+    <col min="2" max="2" width="88" customWidth="1"/>
+    <col min="3" max="3" width="66" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="34" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="17.399999999999999" customHeight="1">
+      <c r="A1" s="4" t="s">
+        <v>363</v>
+      </c>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+    </row>
+    <row r="2" spans="1:5" ht="13.4" customHeight="1">
+      <c r="A2" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+    </row>
+    <row r="3" spans="1:5" ht="58">
+      <c r="A3" s="3" t="s">
+        <v>364</v>
+      </c>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+    </row>
+    <row r="4" spans="1:5" ht="16.649999999999999" customHeight="1">
+      <c r="A4" s="1" t="s">
+        <v>365</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>366</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>378</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>379</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" s="2" t="s">
+        <v>380</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>381</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>382</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>383</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>385</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>386</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>383</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" s="2" t="s">
+        <v>387</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>388</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>383</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" s="2" t="s">
+        <v>391</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>392</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>383</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="25">
+      <c r="A12" s="2" t="s">
+        <v>394</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>396</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>399</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>400</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>383</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="A14" s="2" t="s">
+        <v>402</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>403</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>404</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
+      <c r="A15" s="2" t="s">
+        <v>406</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>383</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="25">
+      <c r="A16" s="2" t="s">
+        <v>409</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>411</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
+      <c r="A17" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>383</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>416</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
+      <c r="A19" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>420</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>383</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5">
+      <c r="A20" s="2" t="s">
+        <v>422</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>383</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5">
+      <c r="A21" s="2" t="s">
+        <v>425</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>427</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>383</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="25">
+      <c r="A22" s="2" t="s">
+        <v>428</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>429</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>383</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5">
+      <c r="A23" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>433</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>434</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="25">
+      <c r="A24" s="2" t="s">
+        <v>435</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5">
+      <c r="A25" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>439</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>383</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5">
+      <c r="A26" s="2" t="s">
+        <v>442</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>443</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>444</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="25">
+      <c r="A27" s="2" t="s">
+        <v>445</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>446</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>447</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="25">
+      <c r="A28" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>449</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>383</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:E2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>